<commit_message>
Update document templates and self-declaration database.
Refresh certificate docx formats, update 自我宣告.xlsx with new items, and remove obsolete duplicate templates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/資料庫&文件範本/自我宣告.xlsx
+++ b/資料庫&文件範本/自我宣告.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://acticloud-my.sharepoint.com/personal/violet_su_acti_com/Documents/文件/Cursor/ACTi_Doc_Generator/資料庫&amp;文件範本/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="8_{43ECBEC5-9D13-42CA-BDEE-238C4138FB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69057625-C80D-431A-A283-537BCD559BAD}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="8_{43ECBEC5-9D13-42CA-BDEE-238C4138FB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{604266EE-00CB-4D00-AE72-A105DE671145}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{E21F4961-F369-4CE3-8703-0540D48C95F4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E21F4961-F369-4CE3-8703-0540D48C95F4}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>宣告</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -123,6 +123,36 @@
     <t>美國 NDAA國防授權法案（National Defense Authorization Act）
 本產品的供應鏈管理流程遵循 NDAA 法規規範，包含材料追溯、製造來源控管及文件審查，確保最終設備可於政府、軍用與所有需符合法規的專案中安心部署。</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>本產品具備完整防塵設計，能有效防止灰塵進入內部（依據 IEC 60529 之等級 6），並可承受最深 1 公尺、最長 30 分鐘之水下浸泡（等級 7），在惡劣環境中亦可穩定運作。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>本產品具備完整防塵設計，能有效防止灰塵進入內部（依據 IEC 60529 之等級 6），並可防止高壓水柱噴射侵入（等級 6），在惡劣環境中亦可穩定運作。</t>
+  </si>
+  <si>
+    <t>The products we provide conform to the essential requirements and relevant provisions of the applicable European Union directives and regulations. All items have undergone the necessary conformity assessment procedures, and the CE marking has been affixed accordingly to indicate compliance with EU safety, health, and environmental protection standards.</t>
+  </si>
+  <si>
+    <t>The products we supply comply with the Federal Communications Commission (FCC) regulations. They meet the applicable requirements under Part 15 of the FCC Rules, ensuring that the equipment does not cause harmful interference and accepts any interference received, including interference that may cause undesired operation.</t>
+  </si>
+  <si>
+    <t>This product is rated IP68 under the IEC 60529 standard, which means it is fully protected against dust ingress and can withstand continuous immersion in water beyond 1 meter depth under manufacturer-defined conditions. It ensures long-term durability in extreme outdoor or industrial environments.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>This product is rated IK10 according to IEC 62262, indicating the highest level of mechanical impact protection. It can withstand an impact energy of 20 joules, equivalent to the impact of a 5 kg mass dropped from a height of 400 mm, making it highly resistant to vandalism or physical tampering.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>This product complies with the requirements set by the Bureau of Standards, Metrology and Inspection (BSMI), Ministry of Economic Affairs, Taiwan. It has passed inspection for electrical safety, electromagnetic compatibility, and labeling requirements. The BSMI certification ensures the product is safe and compliant for sale and use in the Taiwan market.</t>
+  </si>
+  <si>
+    <t>This product aligns with the technical specifications and interoperability standards issued by the Taiwan Association of Information and Communication Standards (TAICS). Compliance with TAICS standards ensures compatibility, reliability, and integration within Taiwan’s ICT infrastructure.</t>
+  </si>
+  <si>
+    <t>The products we provide do not contain, use, or integrate any covered telecommunications equipment or services from prohibited entities as defined under Section 889 of the National Defense Authorization Act (NDAA).</t>
   </si>
 </sst>
 </file>
@@ -168,11 +198,8 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -534,6 +561,9 @@
       <c r="B2" t="s">
         <v>18</v>
       </c>
+      <c r="C2" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -542,16 +572,25 @@
       <c r="B3" t="s">
         <v>17</v>
       </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -560,6 +599,9 @@
       <c r="B6" t="s">
         <v>16</v>
       </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -568,11 +610,17 @@
       <c r="B7" t="s">
         <v>15</v>
       </c>
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -589,13 +637,19 @@
       <c r="B10" t="s">
         <v>14</v>
       </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>19</v>
+      </c>
+      <c r="C11" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>